<commit_message>
feat(map-routing): real HCMC street-graph + OSRM GeoJSON polylines, 15-district dispersed samples, and Gillett-Miller Angular Sweep VRPTW (CR: CR-20261027-001)
</commit_message>
<xml_diff>
--- a/apps/landing/public/samples/EcoMiles_Mau_Chuoi_Lanh_120_Don_Cam_Tai_QD23.xlsx
+++ b/apps/landing/public/samples/EcoMiles_Mau_Chuoi_Lanh_120_Don_Cam_Tai_QD23.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="orders" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Doi_Xe_Hien_Co" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -494,14 +495,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>22 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>22 Ngô Gia Tự, Phường 4, Quận 10, TP.HCM</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>10.759599</v>
+        <v>10.765736</v>
       </c>
       <c r="D2" t="n">
-        <v>106.670888</v>
+        <v>106.670684</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -545,14 +546,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>39 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>39 Hòa Bình, P. Hiệp Tân, Tân Phú, TP.HCM</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>10.772549</v>
+        <v>10.769156</v>
       </c>
       <c r="D3" t="n">
-        <v>106.674792</v>
+        <v>106.634009</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -596,14 +597,14 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>56 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>56 Song Hành Xa Lộ Hà Nội, P. Thảo Điền, TP. Thủ Đức, TP.HCM</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>10.805158</v>
+        <v>10.804479</v>
       </c>
       <c r="D4" t="n">
-        <v>106.649179</v>
+        <v>106.738833</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -647,14 +648,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>73 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>73 Ba Tháng Hai, Phường 12, Quận 10, TP.HCM</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10.777967</v>
+        <v>10.772833</v>
       </c>
       <c r="D5" t="n">
-        <v>106.701806</v>
+        <v>106.669194</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -698,14 +699,14 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>90 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>90 Lạc Long Quân, Phường 10, Tân Bình, TP.HCM</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10.75538</v>
+        <v>10.780686</v>
       </c>
       <c r="D6" t="n">
-        <v>106.675288</v>
+        <v>106.646692</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -749,14 +750,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>107 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>107 Nguyễn Thị Thập, P. Tân Phong, Quận 7, TP.HCM</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>10.769399</v>
+        <v>10.740148</v>
       </c>
       <c r="D7" t="n">
-        <v>106.677438</v>
+        <v>106.709856</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -800,14 +801,14 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>124 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>124 Điện Biên Phủ, Phường 4, Quận 3, TP.HCM</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>10.80427</v>
+        <v>10.775194</v>
       </c>
       <c r="D8" t="n">
-        <v>106.649773</v>
+        <v>106.682023</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -851,14 +852,14 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>141 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>141 Bình Tiên, Phường 3, Quận 6, TP.HCM</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>10.777389</v>
+        <v>10.747948</v>
       </c>
       <c r="D9" t="n">
-        <v>106.708534</v>
+        <v>106.651347</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -902,14 +903,14 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>158 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>158 Nguyễn Gia Trí (D2), Phường 25, Bình Thạnh, TP.HCM</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>10.755849</v>
+        <v>10.804836</v>
       </c>
       <c r="D10" t="n">
-        <v>106.671941</v>
+        <v>106.716021</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -953,14 +954,14 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>175 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>175 Đinh Tiên Hoàng, P. Đa Kao, Quận 1, TP.HCM</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>10.767568</v>
+        <v>10.788862</v>
       </c>
       <c r="D11" t="n">
-        <v>106.668513</v>
+        <v>106.6963</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1004,14 +1005,14 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>192 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>192 Hồng Bàng, Phường 11, Quận 5, TP.HCM</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>10.80605</v>
+        <v>10.755764</v>
       </c>
       <c r="D12" t="n">
-        <v>106.644455</v>
+        <v>106.660622</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1055,14 +1056,14 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>209 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>209 Nguyễn Oanh, Phường 17, Gò Vấp, TP.HCM</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>10.774468</v>
+        <v>10.835414</v>
       </c>
       <c r="D13" t="n">
-        <v>106.704889</v>
+        <v>106.67718</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1106,14 +1107,14 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>226 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>226 Lê Lợi, P. Bến Thành, Quận 1, TP.HCM</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>10.756477</v>
+        <v>10.773137</v>
       </c>
       <c r="D14" t="n">
-        <v>106.673847</v>
+        <v>106.698631</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1157,14 +1158,14 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>243 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>243 Ông Ích Khiêm, Phường 10, Quận 11, TP.HCM</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>10.76806</v>
+        <v>10.765019</v>
       </c>
       <c r="D15" t="n">
-        <v>106.669189</v>
+        <v>106.642216</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1208,14 +1209,14 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>260 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>260 Nguyễn Văn Trỗi, Phường 11, Phú Nhuận, TP.HCM</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>10.805974</v>
+        <v>10.79544</v>
       </c>
       <c r="D16" t="n">
-        <v>106.64997</v>
+        <v>106.674686</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1259,14 +1260,14 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>277 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>277 Kha Vạn Cân, P. Linh Đông, TP. Thủ Đức, TP.HCM</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>10.776124</v>
+        <v>10.839244</v>
       </c>
       <c r="D17" t="n">
-        <v>106.707916</v>
+        <v>106.749286</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1310,14 +1311,14 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>294 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>294 Thành Thái, Phường 14, Quận 10, TP.HCM</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>10.75552</v>
+        <v>10.774031</v>
       </c>
       <c r="D18" t="n">
-        <v>106.67486</v>
+        <v>106.661955</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1361,14 +1362,14 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>311 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>311 Tân Kỳ Tân Quý, P. Sơn Kỳ, Tân Phú, TP.HCM</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>10.773632</v>
+        <v>10.802502</v>
       </c>
       <c r="D19" t="n">
-        <v>106.676824</v>
+        <v>106.62496</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1412,14 +1413,14 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>328 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>328 Dương Bá Trạc, Phường 1, Quận 8, TP.HCM</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>10.805768</v>
+        <v>10.747674</v>
       </c>
       <c r="D20" t="n">
-        <v>106.646699</v>
+        <v>106.68764</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1463,14 +1464,14 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>345 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>345 Kỳ Đồng, Phường 9, Quận 3, TP.HCM</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>10.771626</v>
+        <v>10.782504</v>
       </c>
       <c r="D21" t="n">
-        <v>106.70317</v>
+        <v>106.68063</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1514,14 +1515,14 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>362 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>362 Lý Thường Kiệt, Phường 8, Tân Bình, TP.HCM</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>10.749828</v>
+        <v>10.784909</v>
       </c>
       <c r="D22" t="n">
-        <v>106.674569</v>
+        <v>106.654462</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1565,14 +1566,14 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>379 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>379 Hoàng Diệu, Phường 6, Quận 4, TP.HCM</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>10.771318</v>
+        <v>10.761062</v>
       </c>
       <c r="D23" t="n">
-        <v>106.677719</v>
+        <v>106.702946</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1616,14 +1617,14 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>396 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>396 Cách Mạng Tháng 8, Phường 10, Quận 3, TP.HCM</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>10.801382</v>
+        <v>10.78127</v>
       </c>
       <c r="D24" t="n">
-        <v>106.650823</v>
+        <v>106.675959</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1667,14 +1668,14 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>413 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>413 Kinh Dương Vương, Phường 12, Quận 6, TP.HCM</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>10.773014</v>
+        <v>10.750949</v>
       </c>
       <c r="D25" t="n">
-        <v>106.707631</v>
+        <v>106.636058</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1718,14 +1719,14 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>10 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>10 Bạch Đằng, Phường 15, Bình Thạnh, TP.HCM</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>10.750081</v>
+        <v>10.80129</v>
       </c>
       <c r="D26" t="n">
-        <v>106.671311</v>
+        <v>106.701419</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1769,14 +1770,14 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>27 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>27 Cô Giang, P. Cô Giang, Quận 1, TP.HCM</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>10.773202</v>
+        <v>10.765065</v>
       </c>
       <c r="D27" t="n">
-        <v>106.673077</v>
+        <v>106.693761</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1820,14 +1821,14 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>44 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>44 An Dương Vương, Phường 4, Quận 5, TP.HCM</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>10.805217</v>
+        <v>10.761198</v>
       </c>
       <c r="D28" t="n">
-        <v>106.645797</v>
+        <v>106.676751</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1871,14 +1872,14 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>61 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>61 Quang Trung, Phường 10, Gò Vấp, TP.HCM</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>10.773366</v>
+        <v>10.828361</v>
       </c>
       <c r="D29" t="n">
-        <v>106.703252</v>
+        <v>106.671057</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1922,14 +1923,14 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>78 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>78 Lê Thánh Tôn, P. Bến Nghé, Quận 1, TP.HCM</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>10.753844</v>
+        <v>10.777494</v>
       </c>
       <c r="D30" t="n">
-        <v>106.675938</v>
+        <v>106.7043</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1946,12 +1947,12 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -1973,14 +1974,14 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>95 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>95 Nguyễn Tri Phương, Phường 8, Quận 10, TP.HCM</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>10.770725</v>
+        <v>10.761872</v>
       </c>
       <c r="D31" t="n">
-        <v>106.668622</v>
+        <v>106.666035</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1997,12 +1998,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2012,7 +2013,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Hàng lạnh 2-4C; ưu tiên dỡ hàng nhanh</t>
+          <t>BACKHAUL_PICKUP: Nhận hàng thu hồi chiều về kho từ Quận 10</t>
         </is>
       </c>
     </row>
@@ -2024,14 +2025,14 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>112 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>112 Phan Đăng Lưu, Phường 3, Phú Nhuận, TP.HCM</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>10.804602</v>
+        <v>10.801301</v>
       </c>
       <c r="D32" t="n">
-        <v>106.64719</v>
+        <v>106.682797</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -2048,12 +2049,12 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2075,14 +2076,14 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>129 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>129 Phạm Văn Đồng, P. Hiệp Bình Chánh, TP. Thủ Đức, TP.HCM</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>10.769468</v>
+        <v>10.826114</v>
       </c>
       <c r="D33" t="n">
-        <v>106.704673</v>
+        <v>106.722111</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -2099,12 +2100,12 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -2126,14 +2127,14 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>146 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>146 Tô Hiến Thành, Phường 15, Quận 10, TP.HCM</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>10.753557</v>
+        <v>10.779802</v>
       </c>
       <c r="D34" t="n">
-        <v>106.673171</v>
+        <v>106.663715</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -2177,14 +2178,14 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>163 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>163 Lũy Bán Bích, P. Hòa Thạnh, Tân Phú, TP.HCM</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>10.765556</v>
+        <v>10.772918</v>
       </c>
       <c r="D35" t="n">
-        <v>106.672303</v>
+        <v>106.631513</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -2201,12 +2202,12 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2228,14 +2229,14 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>180 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>180 Huỳnh Tấn Phát, P. Bình Thuận, Quận 7, TP.HCM</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>10.799415</v>
+        <v>10.740941</v>
       </c>
       <c r="D36" t="n">
-        <v>106.645747</v>
+        <v>106.725735</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -2252,12 +2253,12 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2279,14 +2280,14 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>197 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>197 Nguyễn Đình Chiểu, Phường 5, Quận 3, TP.HCM</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>10.771644</v>
+        <v>10.77111</v>
       </c>
       <c r="D37" t="n">
-        <v>106.703094</v>
+        <v>106.684306</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -2303,12 +2304,12 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2318,7 +2319,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Hàng lạnh 2-4C; ưu tiên dỡ hàng nhanh</t>
+          <t>BACKHAUL_PICKUP: Nhận hàng thu hồi chiều về kho từ Quận 3</t>
         </is>
       </c>
     </row>
@@ -2330,14 +2331,14 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>214 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>214 Hoàng Văn Thụ, Phường 4, Tân Bình, TP.HCM</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>10.75821</v>
+        <v>10.798591</v>
       </c>
       <c r="D38" t="n">
-        <v>106.672132</v>
+        <v>106.656682</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -2354,12 +2355,12 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2381,14 +2382,14 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>231 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>231 Nguyễn Hữu Cảnh, Phường 22, Bình Thạnh, TP.HCM</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>10.769116</v>
+        <v>10.792357</v>
       </c>
       <c r="D39" t="n">
-        <v>106.673843</v>
+        <v>106.719006</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -2405,12 +2406,12 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -2432,14 +2433,14 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>248 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>248 Nam Kỳ Khởi Nghĩa, Phường 8, Quận 3, TP.HCM</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>10.801152</v>
+        <v>10.788197</v>
       </c>
       <c r="D40" t="n">
-        <v>106.647658</v>
+        <v>106.685347</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -2483,14 +2484,14 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>265 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>265 Hậu Giang, Phường 6, Quận 6, TP.HCM</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>10.773315</v>
+        <v>10.749345</v>
       </c>
       <c r="D41" t="n">
-        <v>106.702105</v>
+        <v>106.64599</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -2507,12 +2508,12 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -2534,14 +2535,14 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>282 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>282 Điện Biên Phủ, Phường 25, Bình Thạnh, TP.HCM</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>10.751585</v>
+        <v>10.800171</v>
       </c>
       <c r="D42" t="n">
-        <v>106.67502</v>
+        <v>106.716607</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -2558,12 +2559,12 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -2585,14 +2586,14 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>299 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>299 Trần Hưng Đạo, P. Cầu Kho, Quận 1, TP.HCM</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>10.768452</v>
+        <v>10.760844</v>
       </c>
       <c r="D43" t="n">
-        <v>106.673159</v>
+        <v>106.688787</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2609,12 +2610,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -2624,7 +2625,7 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>Hàng lạnh 2-4C; ưu tiên dỡ hàng nhanh</t>
+          <t>BACKHAUL_PICKUP: Nhận hàng thu hồi chiều về kho từ Quận 1</t>
         </is>
       </c>
     </row>
@@ -2636,14 +2637,14 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>316 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>316 Trần Hưng Đạo, Phường 2, Quận 5, TP.HCM</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>10.801282</v>
+        <v>10.755938</v>
       </c>
       <c r="D44" t="n">
-        <v>106.652037</v>
+        <v>106.682048</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -2660,12 +2661,12 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -2687,14 +2688,14 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>333 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>333 Phan Văn Trị, Phường 7, Gò Vấp, TP.HCM</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>10.76953</v>
+        <v>10.822134</v>
       </c>
       <c r="D45" t="n">
-        <v>106.707291</v>
+        <v>106.689649</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2711,12 +2712,12 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -2738,14 +2739,14 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>350 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>350 Hai Bà Trưng, P. Tân Định, Quận 1, TP.HCM</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>10.759314</v>
+        <v>10.791945</v>
       </c>
       <c r="D46" t="n">
-        <v>106.671665</v>
+        <v>106.690933</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -2789,14 +2790,14 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>367 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>367 Lý Thường Kiệt, Phường 14, Quận 10, TP.HCM</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>10.7716</v>
+        <v>10.773152</v>
       </c>
       <c r="D47" t="n">
-        <v>106.669853</v>
+        <v>106.656729</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -2813,12 +2814,12 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -2840,14 +2841,14 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>384 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>384 Phan Xích Long, Phường 2, Phú Nhuận, TP.HCM</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>10.798172</v>
+        <v>10.796943</v>
       </c>
       <c r="D48" t="n">
-        <v>106.651327</v>
+        <v>106.690821</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -2864,12 +2865,12 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -2891,14 +2892,14 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>401 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>401 Trần Não, P. An Khánh, TP. Thủ Đức, TP.HCM</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>10.774764</v>
+        <v>10.788808</v>
       </c>
       <c r="D49" t="n">
-        <v>106.707225</v>
+        <v>106.732628</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -2915,12 +2916,12 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -2930,7 +2931,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Hàng lạnh 2-4C; ưu tiên dỡ hàng nhanh</t>
+          <t>BACKHAUL_PICKUP: Nhận hàng thu hồi chiều về kho từ TP. Thủ Đức</t>
         </is>
       </c>
     </row>
@@ -2942,14 +2943,14 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>418 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>418 Sư Vạn Hạnh, Phường 13, Quận 10, TP.HCM</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>10.755862</v>
+        <v>10.77654</v>
       </c>
       <c r="D50" t="n">
-        <v>106.668446</v>
+        <v>106.665503</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -2966,12 +2967,12 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -2993,14 +2994,14 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>15 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>15 Bàu Cát, Phường 14, Tân Bình, TP.HCM</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>10.766075</v>
+        <v>10.789784</v>
       </c>
       <c r="D51" t="n">
-        <v>106.672858</v>
+        <v>106.641691</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -3017,12 +3018,12 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -3044,14 +3045,14 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>32 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>32 Nguyễn Hữu Thọ, P. Tân Hưng, Quận 7, TP.HCM</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>10.806324</v>
+        <v>10.747152</v>
       </c>
       <c r="D52" t="n">
-        <v>106.642649</v>
+        <v>106.700144</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -3095,14 +3096,14 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>49 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>49 Lê Văn Sỹ, Phường 14, Quận 3, TP.HCM</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>10.777415</v>
+        <v>10.790357</v>
       </c>
       <c r="D53" t="n">
-        <v>106.708132</v>
+        <v>106.679618</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -3119,12 +3120,12 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -3146,14 +3147,14 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>66 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>66 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>10.754672</v>
+        <v>10.801159</v>
       </c>
       <c r="D54" t="n">
-        <v>106.676072</v>
+        <v>106.642643</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -3170,12 +3171,12 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -3197,14 +3198,14 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>83 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>83 Lê Quang Định, Phường 14, Bình Thạnh, TP.HCM</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>10.774682</v>
+        <v>10.812538</v>
       </c>
       <c r="D55" t="n">
-        <v>106.670738</v>
+        <v>106.694412</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -3221,12 +3222,12 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -3236,7 +3237,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>Hàng lạnh 2-4C; ưu tiên dỡ hàng nhanh</t>
+          <t>BACKHAUL_PICKUP: Nhận hàng thu hồi chiều về kho từ Bình Thạnh</t>
         </is>
       </c>
     </row>
@@ -3248,14 +3249,14 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>100 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>100 Võ Văn Tần, Phường 6, Quận 3, TP.HCM</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>10.79919</v>
+        <v>10.775869</v>
       </c>
       <c r="D56" t="n">
-        <v>106.646059</v>
+        <v>106.689135</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -3272,12 +3273,12 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -3299,14 +3300,14 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>117 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>117 Hải Thượng Lãn Ông, Phường 10, Quận 5, TP.HCM</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>10.77089</v>
+        <v>10.749869</v>
       </c>
       <c r="D57" t="n">
-        <v>106.700926</v>
+        <v>106.659312</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -3323,12 +3324,12 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -3350,14 +3351,14 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>134 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>134 Xô Viết Nghệ Tĩnh, Phường 21, Bình Thạnh, TP.HCM</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>10.752311</v>
+        <v>10.796704</v>
       </c>
       <c r="D58" t="n">
-        <v>106.67307</v>
+        <v>106.710682</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -3401,14 +3402,14 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>151 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>151 Nguyễn Trãi, P. Nguyễn Cư Trinh, Quận 1, TP.HCM</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>10.773573</v>
+        <v>10.767183</v>
       </c>
       <c r="D59" t="n">
-        <v>106.67076</v>
+        <v>106.686719</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -3425,12 +3426,12 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -3452,14 +3453,14 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>168 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>168 Nguyễn Trãi, Phường 8, Quận 5, TP.HCM</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>10.805409</v>
+        <v>10.756859</v>
       </c>
       <c r="D60" t="n">
-        <v>106.645249</v>
+        <v>106.671876</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -3476,12 +3477,12 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -3503,14 +3504,14 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>185 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>185 Huỳnh Văn Bánh, Phường 17, Phú Nhuận, TP.HCM</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>10.777207</v>
+        <v>10.79289</v>
       </c>
       <c r="D61" t="n">
-        <v>106.702872</v>
+        <v>106.678535</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -3527,12 +3528,12 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -3542,7 +3543,7 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>Hàng lạnh 2-4C; ưu tiên dỡ hàng nhanh</t>
+          <t>BACKHAUL_PICKUP: Nhận hàng thu hồi chiều về kho từ Phú Nhuận</t>
         </is>
       </c>
     </row>
@@ -3554,14 +3555,14 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>202 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>202 Nguyễn Thị Minh Khai, P. Đa Kao, Quận 1, TP.HCM</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>10.754488</v>
+        <v>10.7871</v>
       </c>
       <c r="D62" t="n">
-        <v>106.667966</v>
+        <v>106.699749</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -3578,12 +3579,12 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -3605,14 +3606,14 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>219 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>219 Ngô Gia Tự, Phường 4, Quận 10, TP.HCM</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>10.77157</v>
+        <v>10.764542</v>
       </c>
       <c r="D63" t="n">
-        <v>106.669726</v>
+        <v>106.670088</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -3629,12 +3630,12 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -3656,14 +3657,14 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>236 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>236 Hòa Bình, P. Hiệp Tân, Tân Phú, TP.HCM</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>10.800009</v>
+        <v>10.767831</v>
       </c>
       <c r="D64" t="n">
-        <v>106.644883</v>
+        <v>106.632758</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -3707,14 +3708,14 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>253 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>253 Song Hành Xa Lộ Hà Nội, P. Thảo Điền, TP. Thủ Đức, TP.HCM</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>10.772017</v>
+        <v>10.80293</v>
       </c>
       <c r="D65" t="n">
-        <v>106.703552</v>
+        <v>106.738153</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -3731,12 +3732,12 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3758,14 +3759,14 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>270 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>270 Ba Tháng Hai, Phường 12, Quận 10, TP.HCM</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>10.755784</v>
+        <v>10.771815</v>
       </c>
       <c r="D66" t="n">
-        <v>106.674469</v>
+        <v>106.67043</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -3782,12 +3783,12 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -3809,14 +3810,14 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>287 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>287 Lạc Long Quân, Phường 10, Tân Bình, TP.HCM</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>10.772158</v>
+        <v>10.781031</v>
       </c>
       <c r="D67" t="n">
-        <v>106.675107</v>
+        <v>106.64641</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -3833,12 +3834,12 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -3848,7 +3849,7 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>Hàng lạnh 2-4C; ưu tiên dỡ hàng nhanh</t>
+          <t>BACKHAUL_PICKUP: Nhận hàng thu hồi chiều về kho từ Tân Bình</t>
         </is>
       </c>
     </row>
@@ -3860,14 +3861,14 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>304 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>304 Nguyễn Thị Thập, P. Tân Phong, Quận 7, TP.HCM</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>10.803452</v>
+        <v>10.740933</v>
       </c>
       <c r="D68" t="n">
-        <v>106.65184</v>
+        <v>106.709985</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -3884,12 +3885,12 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -3911,14 +3912,14 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>321 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>321 Điện Biên Phủ, Phường 4, Quận 3, TP.HCM</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>10.773377</v>
+        <v>10.774365</v>
       </c>
       <c r="D69" t="n">
-        <v>106.70498</v>
+        <v>106.68161</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -3935,12 +3936,12 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -3962,14 +3963,14 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>338 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>338 Bình Tiên, Phường 3, Quận 6, TP.HCM</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>10.757598</v>
+        <v>10.747695</v>
       </c>
       <c r="D70" t="n">
-        <v>106.672073</v>
+        <v>106.649663</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -4013,14 +4014,14 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>355 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>355 Nguyễn Gia Trí (D2), Phường 25, Bình Thạnh, TP.HCM</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>10.773218</v>
+        <v>10.80537</v>
       </c>
       <c r="D71" t="n">
-        <v>106.670201</v>
+        <v>106.71524</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -4037,12 +4038,12 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -4064,14 +4065,14 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>372 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>372 Đinh Tiên Hoàng, P. Đa Kao, Quận 1, TP.HCM</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>10.797443</v>
+        <v>10.78831</v>
       </c>
       <c r="D72" t="n">
-        <v>106.645162</v>
+        <v>106.697148</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -4088,12 +4089,12 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -4115,14 +4116,14 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>389 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>389 Hồng Bàng, Phường 11, Quận 5, TP.HCM</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>10.776683</v>
+        <v>10.755423</v>
       </c>
       <c r="D73" t="n">
-        <v>106.70781</v>
+        <v>106.662815</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -4139,12 +4140,12 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -4154,7 +4155,7 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>Hàng lạnh 2-4C; ưu tiên dỡ hàng nhanh</t>
+          <t>BACKHAUL_PICKUP: Nhận hàng thu hồi chiều về kho từ Quận 5</t>
         </is>
       </c>
     </row>
@@ -4166,14 +4167,14 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>406 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>406 Nguyễn Oanh, Phường 17, Gò Vấp, TP.HCM</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>10.75776</v>
+        <v>10.836147</v>
       </c>
       <c r="D74" t="n">
-        <v>106.668607</v>
+        <v>106.675554</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -4190,12 +4191,12 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -4217,14 +4218,14 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>423 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>423 Lê Lợi, P. Bến Thành, Quận 1, TP.HCM</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>10.77368</v>
+        <v>10.773618</v>
       </c>
       <c r="D75" t="n">
-        <v>106.676967</v>
+        <v>106.699405</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -4241,12 +4242,12 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -4268,14 +4269,14 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>20 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>20 Ông Ích Khiêm, Phường 10, Quận 11, TP.HCM</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>10.797471</v>
+        <v>10.764319</v>
       </c>
       <c r="D76" t="n">
-        <v>106.651385</v>
+        <v>106.644839</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -4319,14 +4320,14 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>37 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>37 Nguyễn Văn Trỗi, Phường 11, Phú Nhuận, TP.HCM</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>10.775787</v>
+        <v>10.794836</v>
       </c>
       <c r="D77" t="n">
-        <v>106.707846</v>
+        <v>106.675127</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -4343,12 +4344,12 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -4370,14 +4371,14 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>54 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>54 Kha Vạn Cân, P. Linh Đông, TP. Thủ Đức, TP.HCM</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>10.755781</v>
+        <v>10.838814</v>
       </c>
       <c r="D78" t="n">
-        <v>106.673902</v>
+        <v>106.746726</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -4394,12 +4395,12 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -4421,14 +4422,14 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>71 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>71 Thành Thái, Phường 14, Quận 10, TP.HCM</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>10.768922</v>
+        <v>10.773295</v>
       </c>
       <c r="D79" t="n">
-        <v>106.670036</v>
+        <v>106.660188</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -4445,12 +4446,12 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -4460,7 +4461,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>Hàng lạnh 2-4C; ưu tiên dỡ hàng nhanh</t>
+          <t>BACKHAUL_PICKUP: Nhận hàng thu hồi chiều về kho từ Quận 10</t>
         </is>
       </c>
     </row>
@@ -4472,14 +4473,14 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>88 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>88 Tân Kỳ Tân Quý, P. Sơn Kỳ, Tân Phú, TP.HCM</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>10.800911</v>
+        <v>10.801119</v>
       </c>
       <c r="D80" t="n">
-        <v>106.64638</v>
+        <v>106.623538</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -4496,12 +4497,12 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -4523,14 +4524,14 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>105 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>105 Dương Bá Trạc, Phường 1, Quận 8, TP.HCM</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>10.776849</v>
+        <v>10.747476</v>
       </c>
       <c r="D81" t="n">
-        <v>106.700644</v>
+        <v>106.686822</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -4547,12 +4548,12 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -4574,14 +4575,14 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>122 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>122 Kỳ Đồng, Phường 9, Quận 3, TP.HCM</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>10.754781</v>
+        <v>10.783194</v>
       </c>
       <c r="D82" t="n">
-        <v>106.677389</v>
+        <v>106.682365</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -4625,14 +4626,14 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>139 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>139 Lý Thường Kiệt, Phường 8, Tân Bình, TP.HCM</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>10.767821</v>
+        <v>10.785643</v>
       </c>
       <c r="D83" t="n">
-        <v>106.677211</v>
+        <v>106.655084</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -4649,12 +4650,12 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -4676,14 +4677,14 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>156 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>156 Hoàng Diệu, Phường 6, Quận 4, TP.HCM</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>10.807095</v>
+        <v>10.762399</v>
       </c>
       <c r="D84" t="n">
-        <v>106.648258</v>
+        <v>106.701839</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -4700,12 +4701,12 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -4727,14 +4728,14 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>173 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>173 Cách Mạng Tháng 8, Phường 10, Quận 3, TP.HCM</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>10.774351</v>
+        <v>10.781676</v>
       </c>
       <c r="D85" t="n">
-        <v>106.699595</v>
+        <v>106.673486</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -4751,12 +4752,12 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -4766,7 +4767,7 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>Hàng lạnh 2-4C; ưu tiên dỡ hàng nhanh</t>
+          <t>BACKHAUL_PICKUP: Nhận hàng thu hồi chiều về kho từ Quận 3</t>
         </is>
       </c>
     </row>
@@ -4778,14 +4779,14 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>190 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>190 Kinh Dương Vương, Phường 12, Quận 6, TP.HCM</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>10.751621</v>
+        <v>10.750183</v>
       </c>
       <c r="D86" t="n">
-        <v>106.675861</v>
+        <v>106.635876</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -4802,12 +4803,12 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -4829,14 +4830,14 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>207 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>207 Bạch Đằng, Phường 15, Bình Thạnh, TP.HCM</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>10.766583</v>
+        <v>10.801547</v>
       </c>
       <c r="D87" t="n">
-        <v>106.676141</v>
+        <v>106.702741</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -4853,12 +4854,12 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4880,14 +4881,14 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>224 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>224 Cô Giang, P. Cô Giang, Quận 1, TP.HCM</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>10.80124</v>
+        <v>10.763925</v>
       </c>
       <c r="D88" t="n">
-        <v>106.64788</v>
+        <v>106.694018</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -4931,14 +4932,14 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>241 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>241 An Dương Vương, Phường 4, Quận 5, TP.HCM</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>10.771955</v>
+        <v>10.75961</v>
       </c>
       <c r="D89" t="n">
-        <v>106.699653</v>
+        <v>106.675905</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -4955,12 +4956,12 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -4982,14 +4983,14 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>258 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>258 Quang Trung, Phường 10, Gò Vấp, TP.HCM</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>10.75451</v>
+        <v>10.828407</v>
       </c>
       <c r="D90" t="n">
-        <v>106.670765</v>
+        <v>106.670645</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -5006,12 +5007,12 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -5033,14 +5034,14 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>275 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>275 Lê Thánh Tôn, P. Bến Nghé, Quận 1, TP.HCM</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>10.771036</v>
+        <v>10.777971</v>
       </c>
       <c r="D91" t="n">
-        <v>106.673421</v>
+        <v>106.703271</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -5057,12 +5058,12 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -5072,7 +5073,7 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>Hàng lạnh 2-4C; ưu tiên dỡ hàng nhanh</t>
+          <t>BACKHAUL_PICKUP: Nhận hàng thu hồi chiều về kho từ Quận 1</t>
         </is>
       </c>
     </row>
@@ -5084,14 +5085,14 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>292 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>292 Nguyễn Tri Phương, Phường 8, Quận 10, TP.HCM</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>10.806322</v>
+        <v>10.763151</v>
       </c>
       <c r="D92" t="n">
-        <v>106.649118</v>
+        <v>106.668114</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -5108,12 +5109,12 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -5135,14 +5136,14 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>309 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>309 Phan Đăng Lưu, Phường 3, Phú Nhuận, TP.HCM</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>10.773271</v>
+        <v>10.800331</v>
       </c>
       <c r="D93" t="n">
-        <v>106.698724</v>
+        <v>106.681208</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -5159,12 +5160,12 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -5186,14 +5187,14 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>326 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>326 Phạm Văn Đồng, P. Hiệp Bình Chánh, TP. Thủ Đức, TP.HCM</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>10.756656</v>
+        <v>10.828094</v>
       </c>
       <c r="D94" t="n">
-        <v>106.66946</v>
+        <v>106.720827</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -5237,14 +5238,14 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>343 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>343 Tô Hiến Thành, Phường 15, Quận 10, TP.HCM</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>10.768146</v>
+        <v>10.779447</v>
       </c>
       <c r="D95" t="n">
-        <v>106.677967</v>
+        <v>106.665025</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -5261,12 +5262,12 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -5288,14 +5289,14 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>360 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>360 Lũy Bán Bích, P. Hòa Thạnh, Tân Phú, TP.HCM</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>10.804633</v>
+        <v>10.775311</v>
       </c>
       <c r="D96" t="n">
-        <v>106.648036</v>
+        <v>106.632067</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -5312,12 +5313,12 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -5339,14 +5340,14 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>377 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>377 Huỳnh Tấn Phát, P. Bình Thuận, Quận 7, TP.HCM</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>10.776357</v>
+        <v>10.742618</v>
       </c>
       <c r="D97" t="n">
-        <v>106.700594</v>
+        <v>106.725206</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -5363,12 +5364,12 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -5378,7 +5379,7 @@
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>Hàng lạnh 2-4C; ưu tiên dỡ hàng nhanh</t>
+          <t>BACKHAUL_PICKUP: Nhận hàng thu hồi chiều về kho từ Quận 7</t>
         </is>
       </c>
     </row>
@@ -5390,14 +5391,14 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>394 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>394 Nguyễn Đình Chiểu, Phường 5, Quận 3, TP.HCM</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>10.756795</v>
+        <v>10.772438</v>
       </c>
       <c r="D98" t="n">
-        <v>106.675235</v>
+        <v>106.685375</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -5414,12 +5415,12 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -5441,14 +5442,14 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>411 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>411 Hoàng Văn Thụ, Phường 4, Tân Bình, TP.HCM</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>10.769467</v>
+        <v>10.797169</v>
       </c>
       <c r="D99" t="n">
-        <v>106.66896</v>
+        <v>106.655443</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -5465,12 +5466,12 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -5492,14 +5493,14 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>8 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>8 Nguyễn Hữu Cảnh, Phường 22, Bình Thạnh, TP.HCM</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>10.802028</v>
+        <v>10.792777</v>
       </c>
       <c r="D100" t="n">
-        <v>106.643022</v>
+        <v>106.717463</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -5543,14 +5544,14 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>25 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>25 Nam Kỳ Khởi Nghĩa, Phường 8, Quận 3, TP.HCM</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>10.771909</v>
+        <v>10.787895</v>
       </c>
       <c r="D101" t="n">
-        <v>106.698761</v>
+        <v>106.68362</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -5567,12 +5568,12 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -5594,14 +5595,14 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>42 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>42 Hậu Giang, Phường 6, Quận 6, TP.HCM</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>10.752806</v>
+        <v>10.748862</v>
       </c>
       <c r="D102" t="n">
-        <v>106.674391</v>
+        <v>106.647105</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -5618,12 +5619,12 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -5645,14 +5646,14 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>59 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>59 Điện Biên Phủ, Phường 25, Bình Thạnh, TP.HCM</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>10.766966</v>
+        <v>10.800069</v>
       </c>
       <c r="D103" t="n">
-        <v>106.673223</v>
+        <v>106.715807</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -5669,12 +5670,12 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -5684,7 +5685,7 @@
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>Hàng lạnh 2-4C; ưu tiên dỡ hàng nhanh</t>
+          <t>BACKHAUL_PICKUP: Nhận hàng thu hồi chiều về kho từ Bình Thạnh</t>
         </is>
       </c>
     </row>
@@ -5696,14 +5697,14 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>76 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>76 Trần Hưng Đạo, P. Cầu Kho, Quận 1, TP.HCM</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>10.803475</v>
+        <v>10.76194</v>
       </c>
       <c r="D104" t="n">
-        <v>106.647079</v>
+        <v>106.688761</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -5720,12 +5721,12 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -5747,14 +5748,14 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>93 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>93 Trần Hưng Đạo, Phường 2, Quận 5, TP.HCM</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>10.775525</v>
+        <v>10.756752</v>
       </c>
       <c r="D105" t="n">
-        <v>106.701859</v>
+        <v>106.679911</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -5771,12 +5772,12 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -5798,14 +5799,14 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>110 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>110 Phan Văn Trị, Phường 7, Gò Vấp, TP.HCM</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>10.758032</v>
+        <v>10.824534</v>
       </c>
       <c r="D106" t="n">
-        <v>106.676293</v>
+        <v>106.689714</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -5849,14 +5850,14 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>127 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>127 Hai Bà Trưng, P. Tân Định, Quận 1, TP.HCM</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>10.770552</v>
+        <v>10.790517</v>
       </c>
       <c r="D107" t="n">
-        <v>106.670509</v>
+        <v>106.690339</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -5873,12 +5874,12 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -5900,14 +5901,14 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>144 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>144 Lý Thường Kiệt, Phường 14, Quận 10, TP.HCM</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>10.802206</v>
+        <v>10.772834</v>
       </c>
       <c r="D108" t="n">
-        <v>106.643923</v>
+        <v>106.656751</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -5924,12 +5925,12 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
@@ -5951,14 +5952,14 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>161 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>161 Phan Xích Long, Phường 2, Phú Nhuận, TP.HCM</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>10.777595</v>
+        <v>10.799414</v>
       </c>
       <c r="D109" t="n">
-        <v>106.700367</v>
+        <v>106.688434</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -5975,12 +5976,12 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
@@ -5990,7 +5991,7 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>Hàng lạnh 2-4C; ưu tiên dỡ hàng nhanh</t>
+          <t>BACKHAUL_PICKUP: Nhận hàng thu hồi chiều về kho từ Phú Nhuận</t>
         </is>
       </c>
     </row>
@@ -6002,14 +6003,14 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>178 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>178 Trần Não, P. An Khánh, TP. Thủ Đức, TP.HCM</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>10.750476</v>
+        <v>10.787116</v>
       </c>
       <c r="D110" t="n">
-        <v>106.675426</v>
+        <v>106.732436</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -6026,12 +6027,12 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -6053,14 +6054,14 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>195 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>195 Sư Vạn Hạnh, Phường 13, Quận 10, TP.HCM</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>10.772305</v>
+        <v>10.776777</v>
       </c>
       <c r="D111" t="n">
-        <v>106.674967</v>
+        <v>106.667365</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -6077,12 +6078,12 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -6104,14 +6105,14 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>212 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>212 Bàu Cát, Phường 14, Tân Bình, TP.HCM</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>10.803408</v>
+        <v>10.791619</v>
       </c>
       <c r="D112" t="n">
-        <v>106.647565</v>
+        <v>106.641917</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -6155,14 +6156,14 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>229 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>229 Nguyễn Hữu Thọ, P. Tân Hưng, Quận 7, TP.HCM</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>10.77595</v>
+        <v>10.746488</v>
       </c>
       <c r="D113" t="n">
-        <v>106.708472</v>
+        <v>106.703127</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -6179,12 +6180,12 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
@@ -6206,14 +6207,14 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>246 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>246 Lê Văn Sỹ, Phường 14, Quận 3, TP.HCM</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>10.759788</v>
+        <v>10.790796</v>
       </c>
       <c r="D114" t="n">
-        <v>106.669409</v>
+        <v>106.677211</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -6230,12 +6231,12 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
@@ -6257,14 +6258,14 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>263 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>263 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>10.772059</v>
+        <v>10.801699</v>
       </c>
       <c r="D115" t="n">
-        <v>106.674309</v>
+        <v>106.641855</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -6281,12 +6282,12 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
@@ -6296,7 +6297,7 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>Hàng lạnh 2-4C; ưu tiên dỡ hàng nhanh</t>
+          <t>BACKHAUL_PICKUP: Nhận hàng thu hồi chiều về kho từ Tân Bình</t>
         </is>
       </c>
     </row>
@@ -6308,14 +6309,14 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>280 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>280 Lê Quang Định, Phường 14, Bình Thạnh, TP.HCM</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>10.803128</v>
+        <v>10.811529</v>
       </c>
       <c r="D116" t="n">
-        <v>106.650767</v>
+        <v>106.696341</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -6332,12 +6333,12 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
@@ -6359,14 +6360,14 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>297 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>297 Võ Văn Tần, Phường 6, Quận 3, TP.HCM</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>10.775038</v>
+        <v>10.777196</v>
       </c>
       <c r="D117" t="n">
-        <v>106.699316</v>
+        <v>106.688097</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -6383,12 +6384,12 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
@@ -6410,14 +6411,14 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>314 Trần Hưng Đạo, Phường 7, Quận 5, TP.HCM</t>
+          <t>314 Hải Thượng Lãn Ông, Phường 10, Quận 5, TP.HCM</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>10.757984</v>
+        <v>10.751819</v>
       </c>
       <c r="D118" t="n">
-        <v>106.669385</v>
+        <v>106.659203</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -6461,14 +6462,14 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>331 Ba Tháng Hai, Phường 11, Quận 10, TP.HCM</t>
+          <t>331 Xô Viết Nghệ Tĩnh, Phường 21, Bình Thạnh, TP.HCM</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>10.769519</v>
+        <v>10.797186</v>
       </c>
       <c r="D119" t="n">
-        <v>106.675077</v>
+        <v>106.711101</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -6485,12 +6486,12 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
@@ -6512,14 +6513,14 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>348 Cộng Hòa, Phường 13, Tân Bình, TP.HCM</t>
+          <t>348 Nguyễn Trãi, P. Nguyễn Cư Trinh, Quận 1, TP.HCM</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>10.805259</v>
+        <v>10.767211</v>
       </c>
       <c r="D120" t="n">
-        <v>106.64737</v>
+        <v>106.687554</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -6536,12 +6537,12 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
@@ -6563,14 +6564,14 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>365 Nguyễn Huệ, P. Bến Nghé, Quận 1, TP.HCM</t>
+          <t>365 Nguyễn Trãi, Phường 8, Quận 5, TP.HCM</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>10.774647</v>
+        <v>10.756071</v>
       </c>
       <c r="D121" t="n">
-        <v>106.705608</v>
+        <v>106.67311</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -6587,12 +6588,12 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
@@ -6602,7 +6603,333 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>Hàng lạnh 2-4C; ưu tiên dỡ hàng nhanh</t>
+          <t>BACKHAUL_PICKUP: Nhận hàng thu hồi chiều về kho từ Quận 5</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>plate</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>capacity_kg</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>fuel</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>l_per_100km</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>51C-000.01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>van_500</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>500</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>petrol</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>8</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>51C-000.02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>truck_800</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>800</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>diesel</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>51C-000.03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>truck_1000</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>petrol</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>51C-000.04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>truck_1500</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>diesel</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>11</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>51C-000.05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>truck_2000</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>petrol</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>12</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>51C-000.06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>van_500</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>500</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>diesel</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>51C-000.07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>truck_800</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>800</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>petrol</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>51C-000.08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>truck_1000</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>diesel</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>8</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>51C-000.09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>truck_1500</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>petrol</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>10</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>51C-000.10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>truck_2000</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>diesel</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>12</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>ready</t>
         </is>
       </c>
     </row>

</xml_diff>